<commit_message>
Simulador de fundos imobiliarios em Excel - desafio DIO
</commit_message>
<xml_diff>
--- a/simulador-fundos-imobiliarios.xlsx
+++ b/simulador-fundos-imobiliarios.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Galo\simulador-fundos-imobiliarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02ADEAC4-FD1B-4496-86C1-C7F34D30A555}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A5F5B2-C05B-4986-B386-2F48E98CE9A8}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Simulador" sheetId="1" r:id="rId1"/>
@@ -185,9 +185,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -282,6 +282,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -326,9 +333,6 @@
   </cellStyleXfs>
   <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -341,9 +345,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -353,29 +354,17 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -383,6 +372,24 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,6 +669,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-043E-4348-84FE-E09235FD9F88}"/>
                 </c:ext>
@@ -689,6 +697,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-043E-4348-84FE-E09235FD9F88}"/>
                 </c:ext>
@@ -716,6 +725,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000005-043E-4348-84FE-E09235FD9F88}"/>
                 </c:ext>
@@ -743,6 +753,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000007-043E-4348-84FE-E09235FD9F88}"/>
                 </c:ext>
@@ -770,6 +781,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000009-043E-4348-84FE-E09235FD9F88}"/>
                 </c:ext>
@@ -797,6 +809,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000B-043E-4348-84FE-E09235FD9F88}"/>
                 </c:ext>
@@ -869,13 +882,13 @@
                   <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>150</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>200</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>250</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>150</c:v>
@@ -1183,398 +1196,398 @@
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="17" style="18" customWidth="1"/>
+    <col min="3" max="3" width="17" style="13" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="5" width="2" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="9" width="17" style="18" customWidth="1"/>
+    <col min="7" max="9" width="17" style="13" customWidth="1"/>
     <col min="10" max="10" width="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
     </row>
     <row r="3" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
     </row>
     <row r="6" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="F6" s="16" t="s">
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="F6" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="12">
         <v>1000</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="22" t="s">
+      <c r="I7" s="16" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="12">
         <v>10</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <v>2</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="15">
         <f>aporte*$F8*12</f>
         <v>24000</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="15">
         <f>-FV(taxa_mensal,$F8*12,aporte)</f>
         <v>26343.155111119566</v>
       </c>
-      <c r="I8" s="20">
+      <c r="I8" s="15">
         <f>H8*taxa_mensal</f>
         <v>210.74524088895654</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="12">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <v>5</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="15">
         <f>aporte*$F9*12</f>
         <v>60000</v>
       </c>
-      <c r="H9" s="20">
+      <c r="H9" s="15">
         <f>-FV(taxa_mensal,$F9*12,aporte)</f>
         <v>76623.866831880223</v>
       </c>
-      <c r="I9" s="20">
+      <c r="I9" s="15">
         <f>H9*taxa_mensal</f>
         <v>612.99093465504177</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <v>10</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="15">
         <f>aporte*$F10*12</f>
         <v>120000</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="15">
         <f>-FV(taxa_mensal,$F10*12,aporte)</f>
         <v>200217.46940991812</v>
       </c>
-      <c r="I10" s="20">
+      <c r="I10" s="15">
         <f>H10*taxa_mensal</f>
         <v>1601.739755279345</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="F11" s="3">
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="F11" s="2">
         <v>20</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="15">
         <f>aporte*$F11*12</f>
         <v>240000</v>
       </c>
-      <c r="H11" s="20">
+      <c r="H11" s="15">
         <f>-FV(taxa_mensal,$F11*12,aporte)</f>
         <v>721131.21927512833</v>
       </c>
-      <c r="I11" s="20">
+      <c r="I11" s="15">
         <f>H11*taxa_mensal</f>
         <v>5769.0497542010271</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="14">
         <f>-FV(taxa_mensal,prazo_anos*12,aporte)</f>
         <v>200217.46940991812</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="2">
         <v>30</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="15">
         <f>aporte*$F12*12</f>
         <v>360000</v>
       </c>
-      <c r="H12" s="20">
+      <c r="H12" s="15">
         <f>-FV(taxa_mensal,$F12*12,aporte)</f>
         <v>2076413.2313710852</v>
       </c>
-      <c r="I12" s="20">
+      <c r="I12" s="15">
         <f>H12*taxa_mensal</f>
         <v>16611.305850968682</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="14">
         <f>patrimonio*taxa_mensal</f>
         <v>1601.739755279345</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="15">
         <f>aporte*prazo_anos*12</f>
         <v>120000</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="15">
         <f>patrimonio-C14</f>
         <v>80217.469409918122</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="12">
         <v>3500</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="12">
         <v>0.3</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="15">
         <f>salario*pct_sugerido</f>
         <v>1050</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="15">
         <f>(1+taxa_mensal)^12-1</f>
         <v>0.10033869371614701</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="15">
         <f>-FV(taxa_mensal,prazo_anos*12,aporte_sugerido)</f>
         <v>210228.34288041404</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="15">
         <f>C22*taxa_mensal</f>
         <v>1681.8267430433123</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="17" t="s">
-        <v>26</v>
+      <c r="C26" s="12" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="C27" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="11" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="20">
+      <c r="C28" s="15">
         <f t="shared" ref="C28:C33" si="0">VLOOKUP(perfil&amp;"-"&amp;$B28,tab_perfis,4,FALSE())</f>
         <v>0.15</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D28" s="3">
         <f t="shared" ref="D28:D33" si="1">aporte*C28</f>
         <v>150</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C29" s="20">
+      <c r="C29" s="15">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="D29" s="3">
+        <f t="shared" si="1"/>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" s="15">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="D30" s="3">
+        <f t="shared" si="1"/>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="15">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+      <c r="D31" s="3">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C32" s="15">
         <f t="shared" si="0"/>
         <v>0.15</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D32" s="3">
         <f t="shared" si="1"/>
         <v>150</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C30" s="20">
-        <f t="shared" si="0"/>
-        <v>0.2</v>
-      </c>
-      <c r="D30" s="4">
-        <f t="shared" si="1"/>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C31" s="20">
-        <f t="shared" si="0"/>
-        <v>0.25</v>
-      </c>
-      <c r="D31" s="4">
-        <f t="shared" si="1"/>
-        <v>250</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="20">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
-      </c>
-      <c r="D32" s="4">
-        <f t="shared" si="1"/>
-        <v>150</v>
-      </c>
-    </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C33" s="20">
+      <c r="C33" s="15">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="D33" s="4">
+      <c r="D33" s="3">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C34" s="21">
+      <c r="C34" s="23">
         <f>SUM(C28:C33)</f>
         <v>1</v>
       </c>
-      <c r="D34" s="8">
+      <c r="D34" s="24">
         <f>SUM(D28:D33)</f>
         <v>1000</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="4" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1623,337 +1636,337 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="17" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="str">
+      <c r="A3" s="5" t="str">
         <f t="shared" ref="A3:A20" si="0">B3&amp;"-"&amp;C3</f>
         <v>Conservador-Lajes Corporativas</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <v>0.1</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="str">
+      <c r="A4" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Conservador-Shoppings</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>0.05</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Conservador-Galpões Logísticos</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <v>0.15</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Conservador-Papel (CRI)</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>0.4</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="str">
+      <c r="A7" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Conservador-Fundo de Fundos (FOF)</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Conservador-Híbrido</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <v>0.1</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="str">
+      <c r="A9" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Moderado-Lajes Corporativas</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="5">
         <v>0.15</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="str">
+      <c r="A10" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Moderado-Shoppings</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="5">
         <v>0.15</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="str">
+      <c r="A11" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Moderado-Galpões Logísticos</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="5">
         <v>0.2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="str">
+      <c r="A12" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Moderado-Papel (CRI)</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="5">
         <v>0.25</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="str">
+      <c r="A13" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Moderado-Fundo de Fundos (FOF)</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <v>0.15</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="str">
+      <c r="A14" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Moderado-Híbrido</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="5">
         <v>0.1</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="str">
+      <c r="A15" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Arrojado-Lajes Corporativas</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="5">
         <v>0.15</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="str">
+      <c r="A16" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Arrojado-Shoppings</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="5">
         <v>0.25</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="str">
+      <c r="A17" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Arrojado-Galpões Logísticos</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="5">
         <v>0.25</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="str">
+      <c r="A18" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Arrojado-Papel (CRI)</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="5">
         <v>0.1</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="str">
+      <c r="A19" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Arrojado-Fundo de Fundos (FOF)</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="5">
         <v>0.15</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="str">
+      <c r="A20" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Arrojado-Híbrido</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="5">
         <v>0.1</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="9" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="9">
         <f>SUMIF($B$3:$B$20,C23,$D$3:$D$20)</f>
         <v>1.0000000000000002</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="9">
         <f>SUMIF($B$3:$B$20,C24,$D$3:$D$20)</f>
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="9">
         <f>SUMIF($B$3:$B$20,C25,$D$3:$D$20)</f>
         <v>1</v>
       </c>

</xml_diff>